<commit_message>
Updated map data to include PFAS chemicals and de-aggregate the chemical data for chemical-specific visualization
</commit_message>
<xml_diff>
--- a/data/TSCA Fenceline Map Chem Hazard Data Extraction_v2.xlsx
+++ b/data/TSCA Fenceline Map Chem Hazard Data Extraction_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edforg.sharepoint.com/sites/SaferChemicals-TSCA/Shared Documents/TSCA/TSCA Fenceline Map Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://edforg-my.sharepoint.com/personal/pvarner_edf_org/Documents/Documents/TSCA/Fenceline Map/TSCA-Map/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1381" documentId="8_{7308D487-D18C-4C8C-8284-D91F0EC2548C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{853155B3-5CEB-4FFB-A809-038CE92E8C24}"/>
+  <xr:revisionPtr revIDLastSave="1508" documentId="8_{7308D487-D18C-4C8C-8284-D91F0EC2548C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C846C3A-933F-4943-A6D6-5A58FED0DF95}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{7FEFC3C9-9C83-49AD-90A9-4B598C07F3FD}"/>
+    <workbookView xWindow="-18450" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{7FEFC3C9-9C83-49AD-90A9-4B598C07F3FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Complete data" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="228">
   <si>
     <t>Carcinogens (15)</t>
   </si>
@@ -604,12 +604,6 @@
     <t>Acute NOAEL (ATSDR)</t>
   </si>
   <si>
-    <t>Convert ppm to mg/L/day</t>
-  </si>
-  <si>
-    <t>RfC (mg/m3)</t>
-  </si>
-  <si>
     <t>Basis</t>
   </si>
   <si>
@@ -664,9 +658,6 @@
     <t>200 ppm (rat, 6 hr/d, inhalation)</t>
   </si>
   <si>
-    <t>3200 ppm (rat, 6 hr/d, inhalation)</t>
-  </si>
-  <si>
     <t>For calculating weight:</t>
   </si>
   <si>
@@ -679,30 +670,18 @@
     <t>50 mg/kg-d (rat, oral)</t>
   </si>
   <si>
-    <t>3 ppm (rat, 6 hr/d, inhalation)</t>
-  </si>
-  <si>
     <t>142 mg/kg-d (rat, oral)</t>
   </si>
   <si>
     <t>100 ppm (rat, 7 hr/d, inhalation)</t>
   </si>
   <si>
-    <t>300 ppm (rat, 7 hr/d, inhalation)</t>
-  </si>
-  <si>
     <t>*highlighted NOAELs come from EPA risk evaluations, not ATSDR</t>
   </si>
   <si>
     <t>*this value is derived from a LOAEL of 20 ppm because there was no NOAEL included, so assuming the NOAEL is roughly 5x lower than this value</t>
   </si>
   <si>
-    <t>*hazard score based off 2014 TSCA Work Plan Methods Document</t>
-  </si>
-  <si>
-    <t>Note to all from Jeremy: Do not change any names of Chemicals before checking with me first, thank you!</t>
-  </si>
-  <si>
     <t>1,1,2-Trichloroethane (not IARC, NTP, EPA)</t>
   </si>
   <si>
@@ -740,9 +719,6 @@
   </si>
   <si>
     <t>101-14-4</t>
-  </si>
-  <si>
-    <t>40 ppm (rat, 6 hr/d, inhalation)</t>
   </si>
   <si>
     <t>Hazard Score (TSCA Workplan)</t>
@@ -821,6 +797,48 @@
   </si>
   <si>
     <t>Cancer (21 of 28)</t>
+  </si>
+  <si>
+    <t>PFAS</t>
+  </si>
+  <si>
+    <t>335-67-1 (PFOA)</t>
+  </si>
+  <si>
+    <t>no links to asthma in IRIS; ATSDR identified some studies that show an association between PFOA and asthma diagnosis but ultimately determine that the finding is not consistent across studies</t>
+  </si>
+  <si>
+    <t>Multiple</t>
+  </si>
+  <si>
+    <t>1 mg/kg/day (mice, oral)</t>
+  </si>
+  <si>
+    <t>375-95-1 (PFNA)</t>
+  </si>
+  <si>
+    <t>*hazard weight based off 2012 TSCA Work Plan Methods Document for developmental toxicity</t>
+  </si>
+  <si>
+    <t>EPA IRIS, CA EPA - Prop 65, ATSDR MRL</t>
+  </si>
+  <si>
+    <t>*this value is derived from an intermediate NOAEL because there were no adequate acute studies</t>
+  </si>
+  <si>
+    <t>516 mg/kg-day (rat, oral)</t>
+  </si>
+  <si>
+    <t>1 mg/kg-d (rat, oral)</t>
+  </si>
+  <si>
+    <t>240 mg/kg-d (mouse, oral)</t>
+  </si>
+  <si>
+    <t>25 mg/kg-d (rat, oral)</t>
+  </si>
+  <si>
+    <t>IRIS RfC (mg/m3)</t>
   </si>
 </sst>
 </file>
@@ -942,13 +960,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1018,7 +1036,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1094,28 +1112,23 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1134,14 +1147,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1472,7 +1477,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFB21133-9E40-49BC-AC90-9436ADC104E2}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:Q45"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="72.81640625" style="1" customWidth="1"/>
@@ -1489,31 +1494,31 @@
     <col min="12" max="12" width="10.453125" style="1" customWidth="1"/>
     <col min="13" max="13" width="19" style="1" customWidth="1"/>
     <col min="14" max="14" width="46" style="1" customWidth="1"/>
-    <col min="15" max="15" width="33.7265625" style="1" customWidth="1"/>
+    <col min="15" max="15" width="43.6328125" style="1" customWidth="1"/>
     <col min="16" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="39.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="40"/>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="42"/>
+      <c r="A1" s="37"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="39"/>
       <c r="E1" s="4"/>
-      <c r="F1" s="39" t="s">
+      <c r="F1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39" t="s">
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39" t="s">
+      <c r="J1" s="36"/>
+      <c r="K1" s="36"/>
+      <c r="L1" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
+      <c r="M1" s="36"/>
+      <c r="N1" s="36"/>
       <c r="O1" s="10" t="s">
         <v>3</v>
       </c>
@@ -2083,11 +2088,11 @@
       <c r="N14" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="O14" s="43" t="s">
+      <c r="O14" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="P14" s="43"/>
-      <c r="Q14" s="43"/>
+      <c r="P14" s="40"/>
+      <c r="Q14" s="40"/>
     </row>
     <row r="15" spans="1:17" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
@@ -2305,7 +2310,7 @@
       <c r="M19" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="N19" s="38" t="s">
+      <c r="N19" s="31" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2358,7 +2363,7 @@
         <v>91</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>64</v>
@@ -2481,7 +2486,7 @@
       <c r="M23" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="N23" s="38" t="s">
+      <c r="N23" s="31" t="s">
         <v>104</v>
       </c>
     </row>
@@ -3229,16 +3234,16 @@
     </row>
     <row r="41" spans="1:15" ht="58" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>16</v>
@@ -3247,7 +3252,7 @@
         <v>17</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H41" s="5" t="s">
         <v>19</v>
@@ -3265,24 +3270,24 @@
         <v>45</v>
       </c>
       <c r="M41" s="9" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="N41" s="8" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
     </row>
     <row r="42" spans="1:15" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>16</v>
@@ -3291,25 +3296,25 @@
         <v>17</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H42" s="5" t="s">
         <v>19</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="K42" s="8" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="M42" s="9" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="N42" s="9" t="s">
         <v>31</v>
@@ -3317,16 +3322,16 @@
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>206</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>16</v>
@@ -3335,7 +3340,7 @@
         <v>45</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H43" s="5" t="s">
         <v>19</v>
@@ -3361,16 +3366,16 @@
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>16</v>
@@ -3379,7 +3384,7 @@
         <v>17</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H44" s="5" t="s">
         <v>19</v>
@@ -3391,7 +3396,7 @@
         <v>23</v>
       </c>
       <c r="K44" s="5" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="L44" s="1" t="s">
         <v>23</v>
@@ -3405,16 +3410,16 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B45" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>16</v>
@@ -3423,7 +3428,7 @@
         <v>17</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="H45" s="5" t="s">
         <v>19</v>
@@ -3445,6 +3450,53 @@
       </c>
       <c r="N45" s="1" t="s">
         <v>23</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" ht="58" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J46" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="K46" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="L46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N46" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="O46" s="9" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -3469,7 +3521,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24BA2280-8E78-4677-ACEC-F5EEA3413D92}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="53.81640625" customWidth="1"/>
@@ -3480,21 +3532,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="44" t="s">
-        <v>221</v>
-      </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44" t="s">
-        <v>217</v>
-      </c>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44" t="s">
-        <v>218</v>
-      </c>
-      <c r="F1" s="44"/>
+      <c r="A1" s="41" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41" t="s">
+        <v>209</v>
+      </c>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41" t="s">
+        <v>210</v>
+      </c>
+      <c r="F1" s="41"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="30" t="s">
         <v>153</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -3515,7 +3567,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>110</v>
@@ -3575,7 +3627,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>106</v>
@@ -3586,11 +3638,11 @@
       <c r="D6" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="36" t="s">
-        <v>192</v>
-      </c>
-      <c r="F6" s="36" t="s">
-        <v>193</v>
+      <c r="E6" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -3713,11 +3765,11 @@
       <c r="B15" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="37" t="s">
-        <v>195</v>
-      </c>
-      <c r="D15" s="36" t="s">
-        <v>196</v>
+      <c r="C15" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -3727,22 +3779,28 @@
       <c r="B16" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="37" t="s">
-        <v>199</v>
-      </c>
-      <c r="D16" s="36" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C16" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="C17" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>111</v>
       </c>
@@ -3750,44 +3808,52 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B22" s="1" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="1" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" t="s">
         <v>195</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>201</v>
-      </c>
-      <c r="B23" t="s">
-        <v>202</v>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -3806,11 +3872,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C4E7569-6D29-4467-9597-E8DEEB24539B}">
-  <dimension ref="A1:U29"/>
+  <dimension ref="A1:T29"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="51" style="12" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.54296875" style="12" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" style="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.81640625" style="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.453125" style="12" bestFit="1" customWidth="1"/>
@@ -3818,43 +3884,42 @@
     <col min="7" max="7" width="38.1796875" style="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.1796875" style="12" customWidth="1"/>
     <col min="9" max="9" width="31.7265625" style="12" customWidth="1"/>
-    <col min="10" max="10" width="15.453125" style="29" customWidth="1"/>
-    <col min="11" max="11" width="14.1796875" style="12" customWidth="1"/>
-    <col min="12" max="12" width="11.7265625" style="22" customWidth="1"/>
-    <col min="13" max="13" width="11.7265625" style="12" customWidth="1"/>
-    <col min="14" max="14" width="9.1796875" style="12"/>
-    <col min="15" max="15" width="38.1796875" style="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.1796875" style="12"/>
-    <col min="17" max="17" width="12.1796875" style="12" customWidth="1"/>
-    <col min="18" max="18" width="29.7265625" style="13" customWidth="1"/>
-    <col min="19" max="19" width="12.26953125" style="13" customWidth="1"/>
-    <col min="20" max="20" width="14.26953125" style="12" customWidth="1"/>
-    <col min="21" max="16384" width="9.1796875" style="12"/>
+    <col min="10" max="10" width="14.1796875" style="12" customWidth="1"/>
+    <col min="11" max="11" width="11.7265625" style="22" customWidth="1"/>
+    <col min="12" max="12" width="11.7265625" style="12" customWidth="1"/>
+    <col min="13" max="13" width="9.1796875" style="12"/>
+    <col min="14" max="14" width="38.1796875" style="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" style="12"/>
+    <col min="16" max="16" width="15.90625" style="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.7265625" style="13" customWidth="1"/>
+    <col min="18" max="18" width="12.26953125" style="13" customWidth="1"/>
+    <col min="19" max="19" width="14.26953125" style="12" customWidth="1"/>
+    <col min="20" max="16384" width="9.1796875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A1" s="45" t="s">
-        <v>221</v>
-      </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="G1" s="45" t="s">
-        <v>217</v>
-      </c>
-      <c r="H1" s="45"/>
-      <c r="O1" s="45" t="s">
-        <v>218</v>
-      </c>
-      <c r="P1" s="45"/>
-      <c r="Q1" s="45"/>
-      <c r="R1" s="45"/>
-      <c r="S1" s="45"/>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-    </row>
-    <row r="2" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A1" s="35" t="s">
+        <v>213</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="G1" s="35" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="35"/>
+      <c r="N1" s="35" t="s">
+        <v>210</v>
+      </c>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
+      <c r="S1" s="35"/>
+      <c r="T1" s="35"/>
+    </row>
+    <row r="2" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A2" s="14" t="s">
         <v>153</v>
       </c>
@@ -3879,39 +3944,36 @@
       <c r="I2" s="15" t="s">
         <v>156</v>
       </c>
-      <c r="J2" s="31" t="s">
+      <c r="J2" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="K2" s="29" t="s">
+        <v>155</v>
+      </c>
+      <c r="L2" s="15"/>
+      <c r="N2" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="O2" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="P2" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q2" s="15" t="s">
         <v>157</v>
       </c>
-      <c r="K2" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="L2" s="32" t="s">
+      <c r="R2" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="S2" s="23" t="s">
         <v>155</v>
       </c>
-      <c r="M2" s="15"/>
-      <c r="O2" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="P2" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="Q2" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="R2" s="15" t="s">
+      <c r="T2" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="S2" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="T2" s="23" t="s">
-        <v>155</v>
-      </c>
-      <c r="U2" s="14" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>109</v>
       </c>
@@ -3919,10 +3981,10 @@
         <v>110</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E3" s="22">
         <v>0.8</v>
@@ -3934,43 +3996,39 @@
         <v>101</v>
       </c>
       <c r="I3" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J3" s="12">
+        <v>1</v>
+      </c>
+      <c r="K3" s="22">
+        <v>0.6</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="P3" s="12">
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="Q3" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="R3" s="20">
+        <f>LOG10(P3)</f>
+        <v>-2.0457574905606752</v>
+      </c>
+      <c r="S3" s="24">
+        <f>R3*S7</f>
+        <v>0.95151511188868609</v>
+      </c>
+      <c r="T3" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="J3" s="29">
-        <f>(3000*7)/24</f>
-        <v>875</v>
-      </c>
-      <c r="K3" s="12">
-        <v>1</v>
-      </c>
-      <c r="L3" s="22">
-        <v>0.6</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q3" s="12">
-        <v>8.9999999999999993E-3</v>
-      </c>
-      <c r="R3" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="S3" s="20">
-        <f>LOG10(Q3)</f>
-        <v>-2.0457574905606752</v>
-      </c>
-      <c r="T3" s="24">
-        <f>S3*T7</f>
-        <v>0.95151511188868609</v>
-      </c>
-      <c r="U3" s="16" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:20" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>67</v>
       </c>
@@ -3978,10 +4036,10 @@
         <v>68</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E4" s="22">
         <v>0.8</v>
@@ -3993,43 +4051,39 @@
         <v>68</v>
       </c>
       <c r="I4" s="26" t="s">
+        <v>165</v>
+      </c>
+      <c r="J4" s="12">
+        <v>1</v>
+      </c>
+      <c r="K4" s="22">
+        <v>0.6</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="P4" s="12">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="Q4" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="R4" s="20">
+        <f t="shared" ref="R4:R6" si="0">LOG10(P4)</f>
+        <v>-2.1549019599857431</v>
+      </c>
+      <c r="S4" s="24">
+        <f>R4*S7</f>
+        <v>1.0022799813887178</v>
+      </c>
+      <c r="T4" s="16" t="s">
         <v>167</v>
       </c>
-      <c r="J4" s="30">
-        <f>(4*23)/24</f>
-        <v>3.8333333333333335</v>
-      </c>
-      <c r="K4" s="12">
-        <v>1</v>
-      </c>
-      <c r="L4" s="22">
-        <v>0.6</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="P4" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q4" s="12">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="R4" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="S4" s="20">
-        <f t="shared" ref="S4:S6" si="0">LOG10(Q4)</f>
-        <v>-2.1549019599857431</v>
-      </c>
-      <c r="T4" s="24">
-        <f>S4*T7</f>
-        <v>1.0022799813887178</v>
-      </c>
-      <c r="U4" s="16" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>76</v>
       </c>
@@ -4037,10 +4091,10 @@
         <v>77</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E5" s="22">
         <v>0.6</v>
@@ -4052,42 +4106,39 @@
         <v>106</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="J5" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="12">
+        <v>170</v>
+      </c>
+      <c r="J5" s="12">
         <v>3</v>
       </c>
-      <c r="L5" s="22">
+      <c r="K5" s="22">
         <v>1</v>
       </c>
+      <c r="N5" s="2" t="s">
+        <v>125</v>
+      </c>
       <c r="O5" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="P5" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="Q5" s="12">
+      <c r="P5" s="12">
         <v>0.1</v>
       </c>
-      <c r="R5" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="S5" s="13">
+      <c r="Q5" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="R5" s="13">
         <f t="shared" si="0"/>
         <v>-1</v>
       </c>
-      <c r="T5" s="24">
-        <f>S5*T7</f>
+      <c r="S5" s="24">
+        <f>R5*S7</f>
         <v>0.46511627906976744</v>
       </c>
-      <c r="U5" s="16" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+      <c r="T5" s="16" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>105</v>
       </c>
@@ -4098,7 +4149,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E6" s="22">
         <v>1</v>
@@ -4110,43 +4161,39 @@
         <v>75</v>
       </c>
       <c r="I6" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="J6" s="29">
-        <f>(200*6)/24</f>
-        <v>50</v>
-      </c>
-      <c r="K6" s="12">
+        <v>174</v>
+      </c>
+      <c r="J6" s="12">
         <v>1</v>
       </c>
-      <c r="L6" s="22">
+      <c r="K6" s="22">
         <v>0.6</v>
       </c>
-      <c r="O6" s="47" t="s">
-        <v>192</v>
-      </c>
-      <c r="P6" s="47" t="s">
-        <v>193</v>
-      </c>
-      <c r="Q6" s="12">
+      <c r="N6" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="P6" s="12">
         <v>8.9999999999999993E-3</v>
       </c>
-      <c r="R6" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="S6" s="13">
+      <c r="Q6" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="R6" s="13">
         <f t="shared" si="0"/>
         <v>-2.0457574905606752</v>
       </c>
-      <c r="T6" s="24">
-        <f>S6*T7</f>
+      <c r="S6" s="24">
+        <f>R6*S7</f>
         <v>0.95151511188868609</v>
       </c>
-      <c r="U6" s="16" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="T6" s="16" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>74</v>
       </c>
@@ -4157,7 +4204,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E7" s="22">
         <v>1</v>
@@ -4169,28 +4216,24 @@
         <v>13</v>
       </c>
       <c r="I7" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="J7" s="29">
-        <f>(3200*6)/24</f>
-        <v>800</v>
-      </c>
-      <c r="K7" s="12">
+        <v>223</v>
+      </c>
+      <c r="J7" s="12">
         <v>1</v>
       </c>
-      <c r="L7" s="22">
+      <c r="K7" s="22">
         <v>0.6</v>
       </c>
-      <c r="P7" s="1"/>
-      <c r="S7" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="T7" s="12">
+      <c r="O7" s="1"/>
+      <c r="R7" s="21" t="s">
+        <v>175</v>
+      </c>
+      <c r="S7" s="12">
         <f>1/(-2.15)</f>
         <v>-0.46511627906976744</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>62</v>
       </c>
@@ -4198,10 +4241,10 @@
         <v>63</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E8" s="22">
         <v>0.6</v>
@@ -4213,21 +4256,17 @@
         <v>25</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="J8" s="29">
-        <f>(498*6)/24</f>
-        <v>124.5</v>
-      </c>
-      <c r="K8" s="12">
+        <v>176</v>
+      </c>
+      <c r="J8" s="12">
         <v>1</v>
       </c>
-      <c r="L8" s="22">
+      <c r="K8" s="22">
         <v>0.6</v>
       </c>
-      <c r="P8" s="1"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>12</v>
       </c>
@@ -4235,10 +4274,10 @@
         <v>13</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E9" s="22">
         <v>0.6</v>
@@ -4250,20 +4289,17 @@
         <v>39</v>
       </c>
       <c r="I9" s="25" t="s">
-        <v>180</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="K9" s="12">
+        <v>177</v>
+      </c>
+      <c r="J9" s="12">
         <v>3</v>
       </c>
-      <c r="L9" s="22">
+      <c r="K9" s="22">
         <v>1</v>
       </c>
-      <c r="P9" s="1"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
@@ -4271,10 +4307,10 @@
         <v>25</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E10" s="22">
         <v>0.6</v>
@@ -4286,19 +4322,16 @@
         <v>122</v>
       </c>
       <c r="I10" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="J10" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="K10" s="12">
+        <v>178</v>
+      </c>
+      <c r="J10" s="12">
         <v>2</v>
       </c>
-      <c r="L10" s="22">
+      <c r="K10" s="22">
         <v>0.8</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>32</v>
       </c>
@@ -4309,7 +4342,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E11" s="22">
         <v>1</v>
@@ -4321,20 +4354,16 @@
         <v>86</v>
       </c>
       <c r="I11" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="J11" s="29">
-        <f>(3*6)/24</f>
-        <v>0.75</v>
-      </c>
-      <c r="K11" s="12">
+        <v>224</v>
+      </c>
+      <c r="J11" s="12">
         <v>3</v>
       </c>
-      <c r="L11" s="22">
+      <c r="K11" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
@@ -4342,10 +4371,10 @@
         <v>35</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E12" s="22">
         <v>0.6</v>
@@ -4357,19 +4386,16 @@
         <v>55</v>
       </c>
       <c r="I12" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="J12" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="K12" s="12">
+        <v>179</v>
+      </c>
+      <c r="J12" s="12">
         <v>2</v>
       </c>
-      <c r="L12" s="22">
+      <c r="K12" s="22">
         <v>0.8</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>85</v>
       </c>
@@ -4377,10 +4403,10 @@
         <v>86</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E13" s="22">
         <v>0.6</v>
@@ -4392,20 +4418,16 @@
         <v>58</v>
       </c>
       <c r="I13" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="J13" s="29">
-        <f>(100*7)/24</f>
-        <v>29.166666666666668</v>
-      </c>
-      <c r="K13" s="12">
+        <v>180</v>
+      </c>
+      <c r="J13" s="12">
         <v>1</v>
       </c>
-      <c r="L13" s="22">
+      <c r="K13" s="22">
         <v>0.6</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>95</v>
       </c>
@@ -4416,7 +4438,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E14" s="22">
         <v>1</v>
@@ -4428,20 +4450,16 @@
         <v>61</v>
       </c>
       <c r="I14" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="J14" s="29">
-        <f>(300*7)/24</f>
-        <v>87.5</v>
-      </c>
-      <c r="K14" s="12">
+        <v>225</v>
+      </c>
+      <c r="J14" s="12">
         <v>1</v>
       </c>
-      <c r="L14" s="22">
+      <c r="K14" s="22">
         <v>0.6</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
@@ -4449,35 +4467,31 @@
         <v>43</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E15" s="22">
         <v>0.8</v>
       </c>
-      <c r="G15" s="46" t="s">
-        <v>195</v>
-      </c>
-      <c r="H15" s="47" t="s">
-        <v>196</v>
+      <c r="G15" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="I15" s="12" t="s">
-        <v>203</v>
-      </c>
-      <c r="J15" s="29">
-        <f>(40*7)/24</f>
-        <v>11.666666666666666</v>
-      </c>
-      <c r="K15" s="12">
+        <v>226</v>
+      </c>
+      <c r="J15" s="12">
         <v>1</v>
       </c>
-      <c r="L15" s="22">
+      <c r="K15" s="22">
         <v>0.6</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>57</v>
       </c>
@@ -4485,35 +4499,31 @@
         <v>58</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E16" s="22">
         <v>0.8</v>
       </c>
-      <c r="G16" s="46" t="s">
-        <v>199</v>
-      </c>
-      <c r="H16" s="47" t="s">
-        <v>200</v>
+      <c r="G16" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="I16" s="12" t="s">
-        <v>205</v>
-      </c>
-      <c r="J16" s="29">
-        <f>(50*7)/24</f>
-        <v>14.583333333333334</v>
-      </c>
-      <c r="K16" s="12">
+        <v>197</v>
+      </c>
+      <c r="J16" s="12">
         <v>1</v>
       </c>
-      <c r="L16" s="22">
+      <c r="K16" s="22">
         <v>0.6</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -4524,15 +4534,28 @@
         <v>1</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E17" s="22">
         <v>1</v>
       </c>
-      <c r="G17" s="46"/>
-      <c r="H17" s="48"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G17" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="I17" s="34" t="s">
+        <v>218</v>
+      </c>
+      <c r="J17" s="32">
+        <v>3</v>
+      </c>
+      <c r="K17" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>111</v>
       </c>
@@ -4540,136 +4563,148 @@
         <v>112</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E18" s="22">
         <v>0.8</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A19" s="47" t="s">
-        <v>192</v>
-      </c>
-      <c r="B19" s="47" t="s">
-        <v>193</v>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>186</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E19" s="22">
         <v>0.6</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A20" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="B20" s="47" t="s">
-        <v>196</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>170</v>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C20" s="17">
+        <v>1</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E20" s="22">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A21" s="47" t="s">
-        <v>197</v>
-      </c>
-      <c r="B21" s="47" t="s">
-        <v>198</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>191</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E21" s="22">
         <v>0.8</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A22" s="47" t="s">
-        <v>199</v>
-      </c>
-      <c r="B22" s="47" t="s">
-        <v>200</v>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>193</v>
       </c>
       <c r="C22" s="17">
         <v>1</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E22" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A23" s="48" t="s">
-        <v>201</v>
-      </c>
-      <c r="B23" s="48" t="s">
-        <v>202</v>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" t="s">
+        <v>195</v>
       </c>
       <c r="C23" s="17">
         <v>1</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E23" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G24" s="27" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G25" s="28" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="G26" s="12" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A29" s="33" t="s">
-        <v>189</v>
-      </c>
-      <c r="B29" s="25"/>
-      <c r="C29" s="34"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="C24" s="17">
+        <v>1</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="E24" s="22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G26" s="27" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G27" s="28" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G28" s="33" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="G29" s="12" t="s">
+        <v>220</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="G1:H1"/>
-    <mergeCell ref="O1:U1"/>
+    <mergeCell ref="N1:T1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="U3" r:id="rId1" xr:uid="{A1247ADF-532A-4DC3-A9C4-A31C3ED2C13C}"/>
-    <hyperlink ref="U4" r:id="rId2" xr:uid="{CA50102A-9206-47B9-AAA9-80645FA324A8}"/>
-    <hyperlink ref="U5" r:id="rId3" xr:uid="{6A7800F5-41A1-4794-A2CE-24E9C8C3E357}"/>
-    <hyperlink ref="U6" r:id="rId4" xr:uid="{EB3AFED5-92A9-4589-8488-9607C3BFBE9F}"/>
+    <hyperlink ref="T3" r:id="rId1" xr:uid="{A1247ADF-532A-4DC3-A9C4-A31C3ED2C13C}"/>
+    <hyperlink ref="T4" r:id="rId2" xr:uid="{CA50102A-9206-47B9-AAA9-80645FA324A8}"/>
+    <hyperlink ref="T5" r:id="rId3" xr:uid="{6A7800F5-41A1-4794-A2CE-24E9C8C3E357}"/>
+    <hyperlink ref="T6" r:id="rId4" xr:uid="{EB3AFED5-92A9-4589-8488-9607C3BFBE9F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId5"/>
@@ -4987,4 +5022,10 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{fe4574ed-bcfd-4bf0-bde8-43713c3f434f}" enabled="0" method="" siteId="{fe4574ed-bcfd-4bf0-bde8-43713c3f434f}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>